<commit_message>
Block incomplete balance reconciliations and verify original evidence hashes
</commit_message>
<xml_diff>
--- a/templates/synthetic-example/synthetic-model.xlsx
+++ b/templates/synthetic-example/synthetic-model.xlsx
@@ -317,7 +317,7 @@
     <t xml:space="preserve">Balance 2020</t>
   </si>
   <si>
-    <t xml:space="preserve">Debe ser cero</t>
+    <t xml:space="preserve">Debe ser cero; N/D bloquea conciliación</t>
   </si>
   <si>
     <t xml:space="preserve">Balance 2021</t>
@@ -2410,7 +2410,7 @@
         <v>95</v>
       </c>
       <c r="B3" s="2" t="n">
-        <f aca="false">Historicos!G3-Historicos!H3-Historicos!I3</f>
+        <f aca="false">IF(COUNT(Historicos!G3:I3)=3,Historicos!G3-Historicos!H3-Historicos!I3,"N/D")</f>
         <v>0</v>
       </c>
       <c r="C3" s="0" t="s">
@@ -2422,7 +2422,7 @@
         <v>97</v>
       </c>
       <c r="B4" s="2" t="n">
-        <f aca="false">Historicos!G4-Historicos!H4-Historicos!I4</f>
+        <f aca="false">IF(COUNT(Historicos!G4:I4)=3,Historicos!G4-Historicos!H4-Historicos!I4,"N/D")</f>
         <v>0</v>
       </c>
       <c r="C4" s="0" t="s">
@@ -2434,7 +2434,7 @@
         <v>98</v>
       </c>
       <c r="B5" s="2" t="n">
-        <f aca="false">Historicos!G5-Historicos!H5-Historicos!I5</f>
+        <f aca="false">IF(COUNT(Historicos!G5:I5)=3,Historicos!G5-Historicos!H5-Historicos!I5,"N/D")</f>
         <v>0</v>
       </c>
       <c r="C5" s="0" t="s">
@@ -2446,7 +2446,7 @@
         <v>99</v>
       </c>
       <c r="B6" s="2" t="n">
-        <f aca="false">Historicos!G6-Historicos!H6-Historicos!I6</f>
+        <f aca="false">IF(COUNT(Historicos!G6:I6)=3,Historicos!G6-Historicos!H6-Historicos!I6,"N/D")</f>
         <v>0</v>
       </c>
       <c r="C6" s="0" t="s">
@@ -2458,7 +2458,7 @@
         <v>100</v>
       </c>
       <c r="B7" s="2" t="n">
-        <f aca="false">Historicos!G7-Historicos!H7-Historicos!I7</f>
+        <f aca="false">IF(COUNT(Historicos!G7:I7)=3,Historicos!G7-Historicos!H7-Historicos!I7,"N/D")</f>
         <v>0</v>
       </c>
       <c r="C7" s="0" t="s">

</xml_diff>